<commit_message>
data: weekly PubMed update (2026-10-19, 108 articles)
</commit_message>
<xml_diff>
--- a/docs/data/tzuchi_trinetx.xlsx
+++ b/docs/data/tzuchi_trinetx.xlsx
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>資料更新時間 (UTC): 2026-10-12T05:53:36+00:00</t>
+          <t>資料更新時間 (UTC): 2026-10-19T04:37:53+00:00</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21">
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23">
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B25" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -1799,7 +1799,11 @@
           <t>Osteoporosis international : a journal established as result of cooperation between the European Foundation for Osteoporosis and the National Osteoporosis Foundation of the USA</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>37/8/2149-2150</t>
+        </is>
+      </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
           <t>10.1007/s00198-026-08166-4</t>
@@ -1898,13 +1902,13 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Taiwan Primary Aldosteronism Investigation (TAIPAI) study group</t>
+          <t>Chun-Fu Lai</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>PMC全文</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -5528,7 +5532,7 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
@@ -6127,7 +6131,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>41252340</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -6135,47 +6139,39 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dosage Studies in TriNetX: The Importance of Eliminating the Unknown.</t>
+          <t>Osimertinib Versus First-Generation Epidermal Growth Factor Receptor Tyrosine Kinase Inhibitors for Metastatic EGFR-Mutant Non-Small Cell Lung Cancer: A Target Trial Emulation Study of Real-World Survival and Safety Outcomes.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Cerebrovascular diseases (Basel, Switzerland)</t>
+          <t>JCO oncology practice</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>55/5/647-648</t>
+          <t>22/10/1844-1853</t>
         </is>
       </c>
       <c r="F64" s="12" t="inlineStr">
         <is>
-          <t>10.1159/000549585</t>
+          <t>10.1200/OP-25-00788</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Tai-Yung Yi</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+          <t>Ren-Hua Ye</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
-      <c r="K64" s="16" t="inlineStr">
-        <is>
-          <t>PubMed e-mail</t>
+          <t>Cho-Hao Lee</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>末位作者(推定)</t>
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
@@ -6185,34 +6181,34 @@
         </is>
       </c>
       <c r="N64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O64" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>S. Karger AG</t>
+          <t>American Society of Clinical Oncology (ASCO)</t>
         </is>
       </c>
       <c r="Q64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Tai-Yung Yi; Joshua Wang</t>
+          <t>Ren-Hua Ye; Hong-Jie Jhou; Hsin-Yu Chen; Li-Ting Kao; Tina Yi-Jin Hsieh; Yu-Han Chen; Xiaoyi Zhang; Ming-Shen Dai; Ching-Liang Ho; Po-Huang Chen; Cho-Hao Lee</t>
         </is>
       </c>
       <c r="S64" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41252340/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41364874/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>41242897</t>
+          <t>41252340</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -6220,32 +6216,32 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Event timing inaccuracies in a retrospective study of low-dose aspirin and acute pancreatitis.</t>
+          <t>Dosage Studies in TriNetX: The Importance of Eliminating the Unknown.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Pancreatology : official journal of the International Association of Pancreatology (IAP) ... [et al.]</t>
+          <t>Cerebrovascular diseases (Basel, Switzerland)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>26/3/507-508</t>
+          <t>55/5/647-648</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
         <is>
-          <t>10.1016/j.pan.2025.11.006</t>
+          <t>10.1159/000549585</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Hung-Da Chen</t>
+          <t>Tai-Yung Yi</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>台北慈濟醫院; 慈濟大學</t>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6258,15 +6254,15 @@
           <t>台北慈濟醫院</t>
         </is>
       </c>
-      <c r="K65" s="14" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
+      <c r="K65" s="16" t="inlineStr">
+        <is>
+          <t>PubMed e-mail</t>
         </is>
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
-          <t>台北慈濟醫院; 慈濟大學</t>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="N65" t="n">
@@ -6277,27 +6273,27 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Elsevier BV</t>
+          <t>S. Karger AG</t>
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Hung-Da Chen; Joshua Wang</t>
+          <t>Tai-Yung Yi; Joshua Wang</t>
         </is>
       </c>
       <c r="S65" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41242897/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41252340/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>41167602</t>
+          <t>41242897</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -6305,53 +6301,53 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Research Design Concerns in a TriNetX Analysis of Venous Thromboembolism in Pediatric Cystic Fibrosis Patients.</t>
+          <t>Event timing inaccuracies in a retrospective study of low-dose aspirin and acute pancreatitis.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Seminars in thrombosis and hemostasis</t>
+          <t>Pancreatology : official journal of the International Association of Pancreatology (IAP) ... [et al.]</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>52/2/275-276</t>
+          <t>26/3/507-508</t>
         </is>
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
-          <t>10.1055/a-2734-3124</t>
+          <t>10.1016/j.pan.2025.11.006</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Chee-Seng Lee</t>
+          <t>Hung-Da Chen</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
+          <t>台北慈濟醫院; 慈濟大學</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Joshua Wang</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
           <t>台北慈濟醫院</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Joshua Wang</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
-      <c r="K66" s="15" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
+      <c r="K66" s="14" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
         </is>
       </c>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
         <is>
-          <t>台北慈濟醫院</t>
+          <t>台北慈濟醫院; 慈濟大學</t>
         </is>
       </c>
       <c r="N66" t="n">
@@ -6362,27 +6358,27 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Georg Thieme Verlag KG</t>
+          <t>Elsevier BV</t>
         </is>
       </c>
       <c r="Q66" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>Chee-Seng Lee; Joshua Wang</t>
+          <t>Hung-Da Chen; Joshua Wang</t>
         </is>
       </c>
       <c r="S66" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41167602/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41242897/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41167602</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -6390,80 +6386,84 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Psoriatic arthritis risk in psoriasis patients receiving anti-IL-23 vs anti-IL-17: comparison of drug classes and individual agents.</t>
+          <t>Research Design Concerns in a TriNetX Analysis of Venous Thromboembolism in Pediatric Cystic Fibrosis Patients.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Rheumatology (Oxford, England)</t>
+          <t>Seminars in thrombosis and hemostasis</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>65/1</t>
+          <t>52/2/275-276</t>
         </is>
       </c>
       <c r="F67" s="12" t="inlineStr">
         <is>
-          <t>10.1093/rheumatology/keaf489</t>
+          <t>10.1055/a-2734-3124</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Teng-Li Lin</t>
+          <t>Chee-Seng Lee</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>大林慈濟醫院</t>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Yi-Ju Chen; Chun-Ying Wu</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" s="14" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
+          <t>Joshua Wang</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
+      <c r="K67" s="15" t="inlineStr">
+        <is>
+          <t>末位作者(推定)</t>
         </is>
       </c>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
-          <t>大林慈濟醫院</t>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="N67" t="n">
         <v>2</v>
       </c>
       <c r="O67" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Oxford University Press (OUP)</t>
+          <t>Georg Thieme Verlag KG</t>
         </is>
       </c>
       <c r="Q67" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>Teng-Li Lin; Yi-Hsuan Fan; Kuo-Sheng Fan; Chao-Kuei Juan; Yi-Ju Chen; Chun-Ying Wu</t>
+          <t>Chee-Seng Lee; Joshua Wang</t>
         </is>
       </c>
       <c r="S67" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41105233/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41167602/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>41014190</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -6471,44 +6471,40 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Increasing Pediatric Cohort Sizes in TriNetX.</t>
+          <t>Psoriatic arthritis risk in psoriasis patients receiving anti-IL-23 vs anti-IL-17: comparison of drug classes and individual agents.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Journal of burn care &amp; research : official publication of the American Burn Association</t>
+          <t>Rheumatology (Oxford, England)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>47/2/699</t>
+          <t>65/1</t>
         </is>
       </c>
       <c r="F68" s="12" t="inlineStr">
         <is>
-          <t>10.1093/jbcr/iraf186</t>
+          <t>10.1093/rheumatology/keaf489</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Meing-Chung Chang</t>
+          <t>Teng-Li Lin</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>台北慈濟醫院</t>
+          <t>大林慈濟醫院</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+          <t>Yi-Ju Chen; Chun-Ying Wu</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
       <c r="K68" s="14" t="inlineStr">
         <is>
           <t>OpenAlex</t>
@@ -6517,14 +6513,14 @@
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
-          <t>台北慈濟醫院</t>
+          <t>大林慈濟醫院</t>
         </is>
       </c>
       <c r="N68" t="n">
         <v>2</v>
       </c>
       <c r="O68" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P68" t="inlineStr">
         <is>
@@ -6532,23 +6528,23 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Meing-Chung Chang; Joshua Wang</t>
+          <t>Teng-Li Lin; Yi-Hsuan Fan; Kuo-Sheng Fan; Chao-Kuei Juan; Yi-Ju Chen; Chun-Ying Wu</t>
         </is>
       </c>
       <c r="S68" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41014190/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41105233/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41014190</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -6556,38 +6552,42 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>RISK OF AGE-RELATED MACULAR DEGENERATION IN LATE-ONSET ATOPIC DERMATITIS: A Multidatabase Cohort Analysis.</t>
+          <t>Increasing Pediatric Cohort Sizes in TriNetX.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Retina (Philadelphia, Pa.)</t>
+          <t>Journal of burn care &amp; research : official publication of the American Burn Association</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>46/1/136-145</t>
+          <t>47/2/699</t>
         </is>
       </c>
       <c r="F69" s="12" t="inlineStr">
         <is>
-          <t>10.1097/IAE.0000000000004634</t>
+          <t>10.1093/jbcr/iraf186</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Tai-Li Chen</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr"/>
+          <t>Meing-Chung Chang</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Tai-Li Chen; Hou-Ren Tsai</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>花蓮慈濟醫院; 慈濟大學</t>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="K69" s="14" t="inlineStr">
@@ -6598,103 +6598,99 @@
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
-          <t>花蓮慈濟醫院; 慈濟大學</t>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="N69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O69" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Ovid Technologies (Wolters Kluwer Health)</t>
+          <t>Oxford University Press (OUP)</t>
         </is>
       </c>
       <c r="Q69" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Tai-Li Chen; Hou-Ren Tsai; Wei-Chuan Chang; Jing-Wun Lu; Yi-Ju Chen; Yuan-Chieh Lee; Chen-Yi Wu</t>
+          <t>Meing-Chung Chang; Joshua Wang</t>
         </is>
       </c>
       <c r="S69" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/40729752/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41014190/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Prognostic implications of serum ferritin levels in non-anemic women with stage 3 chronic kidney disease.</t>
+          <t>RISK OF AGE-RELATED MACULAR DEGENERATION IN LATE-ONSET ATOPIC DERMATITIS: A Multidatabase Cohort Analysis.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Frontiers in nutrition</t>
+          <t>Retina (Philadelphia, Pa.)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>12/1682003</t>
+          <t>46/1/136-145</t>
         </is>
       </c>
       <c r="F70" s="12" t="inlineStr">
         <is>
-          <t>10.3389/fnut.2025.1682003</t>
+          <t>10.1097/IAE.0000000000004634</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Min-Tser Liao</t>
+          <t>Tai-Li Chen</t>
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Kuo-Cheng Lu</t>
+          <t>Tai-Li Chen; Hou-Ren Tsai</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
-      <c r="K70" s="13" t="inlineStr">
-        <is>
-          <t>PMC全文</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>一致</t>
-        </is>
-      </c>
+          <t>花蓮慈濟醫院; 慈濟大學</t>
+        </is>
+      </c>
+      <c r="K70" s="14" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
-          <t>台北慈濟醫院; 花蓮慈濟醫院; 慈濟大學</t>
+          <t>花蓮慈濟醫院; 慈濟大學</t>
         </is>
       </c>
       <c r="N70" t="n">
         <v>4</v>
       </c>
       <c r="O70" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Frontiers Media SA</t>
+          <t>Ovid Technologies (Wolters Kluwer Health)</t>
         </is>
       </c>
       <c r="Q70" t="n">
@@ -6702,19 +6698,19 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Min-Tser Liao; Chien-Lin Lu; Yi-Chou Hou; Joshua Wang; Kuo-Wang Tsai; Li-Jane Shih; Chia-Chao Wu; Yi-Chun Wang; Kuo-Cheng Lu</t>
+          <t>Tai-Li Chen; Hou-Ren Tsai; Wei-Chuan Chang; Jing-Wun Lu; Yi-Ju Chen; Yuan-Chieh Lee; Chen-Yi Wu</t>
         </is>
       </c>
       <c r="S70" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41445831/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/40729752/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>41427560</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -6722,52 +6718,64 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Letter to the Editor: Design Concerns in a TriNetX-Based Study of ACL Reconstruction Outcomes.</t>
+          <t>Prognostic implications of serum ferritin levels in non-anemic women with stage 3 chronic kidney disease.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Journal of pediatric orthopedics</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr"/>
+          <t>Frontiers in nutrition</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>12/1682003</t>
+        </is>
+      </c>
       <c r="F71" s="12" t="inlineStr">
         <is>
-          <t>10.1097/BPO.0000000000003170</t>
+          <t>10.3389/fnut.2025.1682003</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Kuen-Huei Lin</t>
+          <t>Min-Tser Liao</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Kuen-Huei Lin</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" s="14" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr"/>
+          <t>Kuo-Cheng Lu</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
+      <c r="K71" s="13" t="inlineStr">
+        <is>
+          <t>PMC全文</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>一致</t>
+        </is>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>台北慈濟醫院</t>
+          <t>台北慈濟醫院; 花蓮慈濟醫院; 慈濟大學</t>
         </is>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O71" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Ovid Technologies (Wolters Kluwer Health)</t>
+          <t>Frontiers Media SA</t>
         </is>
       </c>
       <c r="Q71" t="n">
@@ -6775,19 +6783,19 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Kuen-Huei Lin; Joshua Wang</t>
+          <t>Min-Tser Liao; Chien-Lin Lu; Yi-Chou Hou; Joshua Wang; Kuo-Wang Tsai; Li-Jane Shih; Chia-Chao Wu; Yi-Chun Wang; Kuo-Cheng Lu</t>
         </is>
       </c>
       <c r="S71" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41427560/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41445831/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41427560</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -6795,39 +6803,35 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Osimertinib Versus First-Generation Epidermal Growth Factor Receptor Tyrosine Kinase Inhibitors for Metastatic EGFR-Mutant Non-Small Cell Lung Cancer: A Target Trial Emulation Study of Real-World Survival and Safety Outcomes.</t>
+          <t>Letter to the Editor: Design Concerns in a TriNetX-Based Study of ACL Reconstruction Outcomes.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>JCO oncology practice</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>OP2500788</t>
-        </is>
-      </c>
+          <t>Journal of pediatric orthopedics</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
       <c r="F72" s="12" t="inlineStr">
         <is>
-          <t>10.1200/OP-25-00788</t>
+          <t>10.1097/BPO.0000000000003170</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Ren-Hua Ye</t>
+          <t>Kuen-Huei Lin</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Cho-Hao Lee</t>
+          <t>Kuen-Huei Lin</t>
         </is>
       </c>
       <c r="J72" t="inlineStr"/>
-      <c r="K72" s="15" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
+      <c r="K72" s="14" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
         </is>
       </c>
       <c r="L72" t="inlineStr"/>
@@ -6840,11 +6844,11 @@
         <v>1</v>
       </c>
       <c r="O72" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>American Society of Clinical Oncology (ASCO)</t>
+          <t>Ovid Technologies (Wolters Kluwer Health)</t>
         </is>
       </c>
       <c r="Q72" t="n">
@@ -6852,12 +6856,12 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Ren-Hua Ye; Hong-Jie Jhou; Hsin-Yu Chen; Li-Ting Kao; Tina Yi-Jin Hsieh; Yu-Han Chen; Xiaoyi Zhang; Ming-Shen Dai; Ching-Liang Ho; Po-Huang Chen; Cho-Hao Lee</t>
+          <t>Kuen-Huei Lin; Joshua Wang</t>
         </is>
       </c>
       <c r="S72" s="12" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/41364874/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41427560/</t>
         </is>
       </c>
     </row>
@@ -9864,7 +9868,7 @@
         </is>
       </c>
       <c r="Q108" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="R108" t="inlineStr">
         <is>
@@ -12664,9 +12668,21 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>PMC全文</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
@@ -12728,16 +12744,8 @@
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
-        </is>
-      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
@@ -25892,7 +25900,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>41252340</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B385" t="n">
@@ -25903,10 +25911,14 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>Tai-Yung Yi</t>
-        </is>
-      </c>
-      <c r="E385" t="inlineStr"/>
+          <t>Ren-Hua Ye</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>0000-0003-2418-7829</t>
+        </is>
+      </c>
       <c r="F385" t="inlineStr">
         <is>
           <t>Y</t>
@@ -25916,67 +25928,55 @@
       <c r="H385" t="inlineStr"/>
       <c r="I385" t="inlineStr"/>
       <c r="J385" t="inlineStr"/>
-      <c r="K385" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K385" t="inlineStr"/>
       <c r="L385" t="inlineStr">
         <is>
-          <t>Department of Pharmacy, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>41252340</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B386" t="n">
         <v>2026</v>
       </c>
       <c r="C386" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Ren-Hua Ye</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
-        </is>
-      </c>
-      <c r="F386" t="inlineStr"/>
-      <c r="G386" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H386" t="inlineStr">
-        <is>
-          <t>PubMed e-mail</t>
-        </is>
-      </c>
+          <t>0000-0003-2418-7829</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr"/>
+      <c r="H386" t="inlineStr"/>
       <c r="I386" t="inlineStr"/>
       <c r="J386" t="inlineStr"/>
-      <c r="K386" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K386" t="inlineStr"/>
       <c r="L386" t="inlineStr">
         <is>
-          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan, reillyjj@qut.edu.au.</t>
+          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>41252340</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B387" t="n">
@@ -25987,195 +25987,151 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Hong-Jie Jhou</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
+          <t>0000-0003-3304-4643</t>
         </is>
       </c>
       <c r="F387" t="inlineStr"/>
-      <c r="G387" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H387" t="inlineStr">
-        <is>
-          <t>PubMed e-mail</t>
-        </is>
-      </c>
+      <c r="G387" t="inlineStr"/>
+      <c r="H387" t="inlineStr"/>
       <c r="I387" t="inlineStr"/>
       <c r="J387" t="inlineStr"/>
       <c r="K387" t="inlineStr"/>
       <c r="L387" t="inlineStr">
         <is>
-          <t>School of Biomedical Sciences, Queensland University of Technology, Brisbane, Queensland, Australia, reillyjj@qut.edu.au.</t>
+          <t>Neurological Institute, Changhua Christian Hospital, Changhua, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>41242897</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B388" t="n">
         <v>2026</v>
       </c>
       <c r="C388" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>Hung-Da Chen</t>
+          <t>Hsin-Yu Chen</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>0009-0000-0327-8663</t>
-        </is>
-      </c>
-      <c r="F388" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>0000-0002-2765-1685</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr"/>
       <c r="G388" t="inlineStr"/>
       <c r="H388" t="inlineStr"/>
       <c r="I388" t="inlineStr"/>
       <c r="J388" t="inlineStr"/>
-      <c r="K388" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院; 慈濟大學</t>
-        </is>
-      </c>
+      <c r="K388" t="inlineStr"/>
       <c r="L388" t="inlineStr">
         <is>
-          <t>Division of Gastroenterology, Department of Internal Medicine, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan; College of Medicine, Tzu Chi University, Hualien, Taiwan.</t>
+          <t>Department of Family Medicine, Chi Mei Medical Center, Tainan, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>41242897</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B389" t="n">
         <v>2026</v>
       </c>
       <c r="C389" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Li-Ting Kao</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
+          <t>0000-0003-0692-7408</t>
         </is>
       </c>
       <c r="F389" t="inlineStr"/>
-      <c r="G389" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H389" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+      <c r="G389" t="inlineStr"/>
+      <c r="H389" t="inlineStr"/>
       <c r="I389" t="inlineStr"/>
-      <c r="J389" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K389" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="J389" t="inlineStr"/>
+      <c r="K389" t="inlineStr"/>
       <c r="L389" t="inlineStr">
         <is>
-          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan; School of Biomedical Sciences, Queensland University of Technology, Brisbane, Australia. Electronic address: reillyjj@qut.edu.au.</t>
+          <t>Graduate Institute of Life Sciences, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>41167602</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B390" t="n">
         <v>2026</v>
       </c>
       <c r="C390" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Chee-Seng Lee</t>
+          <t>Li-Ting Kao</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>0000-0002-3681-7288</t>
-        </is>
-      </c>
-      <c r="F390" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>0000-0003-0692-7408</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr"/>
       <c r="H390" t="inlineStr"/>
       <c r="I390" t="inlineStr"/>
       <c r="J390" t="inlineStr"/>
-      <c r="K390" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K390" t="inlineStr"/>
       <c r="L390" t="inlineStr">
         <is>
-          <t>Department of Pediatrics, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>School of Pharmacy, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>41167602</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B391" t="n">
         <v>2026</v>
       </c>
       <c r="C391" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>Chee-Seng Lee</t>
+          <t>Li-Ting Kao</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>0000-0002-3681-7288</t>
-        </is>
-      </c>
-      <c r="F391" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>0000-0003-0692-7408</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr"/>
       <c r="H391" t="inlineStr"/>
       <c r="I391" t="inlineStr"/>
@@ -26183,167 +26139,135 @@
       <c r="K391" t="inlineStr"/>
       <c r="L391" t="inlineStr">
         <is>
-          <t>Department of Pediatrics, National Taiwan University Children's Hospital, Taipei, Taiwan.</t>
+          <t>Department of Pharmacy Practice, Tri-Service General Hospital, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>41167602</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B392" t="n">
         <v>2026</v>
       </c>
       <c r="C392" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Tina Yi-Jin Hsieh</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
+          <t>0000-0001-6296-0689</t>
         </is>
       </c>
       <c r="F392" t="inlineStr"/>
-      <c r="G392" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H392" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
-        </is>
-      </c>
+      <c r="G392" t="inlineStr"/>
+      <c r="H392" t="inlineStr"/>
       <c r="I392" t="inlineStr"/>
       <c r="J392" t="inlineStr"/>
-      <c r="K392" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K392" t="inlineStr"/>
       <c r="L392" t="inlineStr">
         <is>
-          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>Department of Obstetrics and Gynecology, Beth Israel Deaconess Medical Center, Boston, MA.</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>41167602</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B393" t="n">
         <v>2026</v>
       </c>
       <c r="C393" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Yu-Han Chen</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
+          <t>0000-0001-9170-7439</t>
         </is>
       </c>
       <c r="F393" t="inlineStr"/>
-      <c r="G393" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H393" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
-        </is>
-      </c>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr"/>
       <c r="I393" t="inlineStr"/>
       <c r="J393" t="inlineStr"/>
       <c r="K393" t="inlineStr"/>
       <c r="L393" t="inlineStr">
         <is>
-          <t>School of Biomedical Sciences, Queensland University of Technology, Brisbane, Australia.</t>
+          <t>Department of Internal Medicine, Englewood Hospital and Medical Center, Englewood, NJ.</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B394" t="n">
         <v>2026</v>
       </c>
       <c r="C394" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>Teng-Li Lin</t>
+          <t>Xiaoyi Zhang</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>0000-0002-0639-3533</t>
-        </is>
-      </c>
-      <c r="F394" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>0000-0001-5124-4919</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr"/>
       <c r="G394" t="inlineStr"/>
       <c r="H394" t="inlineStr"/>
       <c r="I394" t="inlineStr"/>
       <c r="J394" t="inlineStr"/>
-      <c r="K394" s="19" t="inlineStr">
-        <is>
-          <t>大林慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K394" t="inlineStr"/>
       <c r="L394" t="inlineStr">
         <is>
-          <t>Department of Dermatology, Dalin Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Chiayi, Taiwan.</t>
+          <t>Department of Internal Medicine, NYC Health + Hospitals/Jacobi, Albert Einstein College of Medicine, Bronx, NY.</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B395" t="n">
         <v>2026</v>
       </c>
       <c r="C395" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>Teng-Li Lin</t>
+          <t>Ming-Shen Dai</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>0000-0002-0639-3533</t>
-        </is>
-      </c>
-      <c r="F395" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>0000-0002-3953-5243</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr"/>
       <c r="G395" t="inlineStr"/>
       <c r="H395" t="inlineStr"/>
       <c r="I395" t="inlineStr"/>
@@ -26351,28 +26275,32 @@
       <c r="K395" t="inlineStr"/>
       <c r="L395" t="inlineStr">
         <is>
-          <t>Ph.D. Program of Interdisciplinary Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
+          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B396" t="n">
         <v>2026</v>
       </c>
       <c r="C396" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>Yi-Hsuan Fan</t>
-        </is>
-      </c>
-      <c r="E396" t="inlineStr"/>
+          <t>Ming-Shen Dai</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>0000-0002-3953-5243</t>
+        </is>
+      </c>
       <c r="F396" t="inlineStr"/>
       <c r="G396" t="inlineStr"/>
       <c r="H396" t="inlineStr"/>
@@ -26381,64 +26309,64 @@
       <c r="K396" t="inlineStr"/>
       <c r="L396" t="inlineStr">
         <is>
-          <t>Department of Pediatrics, Chung Shan Medical University Hospital, Taichung, Taiwan.</t>
+          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B397" t="n">
         <v>2026</v>
       </c>
       <c r="C397" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>Kuo-Sheng Fan</t>
-        </is>
-      </c>
-      <c r="E397" t="inlineStr"/>
+          <t>Ching-Liang Ho</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>0000-0002-8378-1687</t>
+        </is>
+      </c>
       <c r="F397" t="inlineStr"/>
       <c r="G397" t="inlineStr"/>
       <c r="H397" t="inlineStr"/>
       <c r="I397" t="inlineStr"/>
       <c r="J397" t="inlineStr"/>
-      <c r="K397" s="19" t="inlineStr">
-        <is>
-          <t>大林慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K397" t="inlineStr"/>
       <c r="L397" t="inlineStr">
         <is>
-          <t>Division of Chest Medicine, Department of Internal Medicine, Dalin Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Chiayi, Taiwan.</t>
+          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B398" t="n">
         <v>2026</v>
       </c>
       <c r="C398" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>Chao-Kuei Juan</t>
+          <t>Ching-Liang Ho</t>
         </is>
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>0000-0002-8846-0831</t>
+          <t>0000-0002-8378-1687</t>
         </is>
       </c>
       <c r="F398" t="inlineStr"/>
@@ -26449,156 +26377,136 @@
       <c r="K398" t="inlineStr"/>
       <c r="L398" t="inlineStr">
         <is>
-          <t>Department of Dermatology, Taichung Veterans General Hospital, Taichung, Taiwan.</t>
+          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B399" t="n">
         <v>2026</v>
       </c>
       <c r="C399" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>Yi-Ju Chen</t>
-        </is>
-      </c>
-      <c r="E399" t="inlineStr"/>
+          <t>Ching-Liang Ho</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>0000-0002-8378-1687</t>
+        </is>
+      </c>
       <c r="F399" t="inlineStr"/>
-      <c r="G399" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H399" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+      <c r="G399" t="inlineStr"/>
+      <c r="H399" t="inlineStr"/>
       <c r="I399" t="inlineStr"/>
-      <c r="J399" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K399" t="inlineStr"/>
+      <c r="J399" t="inlineStr"/>
+      <c r="K399" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>Department of Dermatology, Taichung Veterans General Hospital, Taichung, Taiwan.</t>
+          <t>Division of Hematology and Oncology, Medical Department, Taipei Tzu Chi Hospital, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B400" t="n">
         <v>2026</v>
       </c>
       <c r="C400" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>Yi-Ju Chen</t>
-        </is>
-      </c>
-      <c r="E400" t="inlineStr"/>
+          <t>Po-Huang Chen</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>0000-0002-0280-6417</t>
+        </is>
+      </c>
       <c r="F400" t="inlineStr"/>
-      <c r="G400" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H400" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+      <c r="G400" t="inlineStr"/>
+      <c r="H400" t="inlineStr"/>
       <c r="I400" t="inlineStr"/>
-      <c r="J400" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J400" t="inlineStr"/>
       <c r="K400" t="inlineStr"/>
       <c r="L400" t="inlineStr">
         <is>
-          <t>Department of Post-Baccalaureate Medicine, National Chung-Hsing University, Taichung, Taiwan.</t>
+          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B401" t="n">
         <v>2026</v>
       </c>
       <c r="C401" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Yi-Ju Chen</t>
-        </is>
-      </c>
-      <c r="E401" t="inlineStr"/>
+          <t>Po-Huang Chen</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>0000-0002-0280-6417</t>
+        </is>
+      </c>
       <c r="F401" t="inlineStr"/>
-      <c r="G401" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H401" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+      <c r="G401" t="inlineStr"/>
+      <c r="H401" t="inlineStr"/>
       <c r="I401" t="inlineStr"/>
-      <c r="J401" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J401" t="inlineStr"/>
       <c r="K401" t="inlineStr"/>
       <c r="L401" t="inlineStr">
         <is>
-          <t>Faculty of Medicine and Institute of Clinical Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
+          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B402" t="n">
         <v>2026</v>
       </c>
       <c r="C402" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Chun-Ying Wu</t>
+          <t>Cho-Hao Lee</t>
         </is>
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>0000-0001-5053-1801</t>
+          <t>0000-0002-6061-5168</t>
         </is>
       </c>
       <c r="F402" t="inlineStr"/>
@@ -26609,42 +26517,38 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>OpenAlex</t>
+          <t>末位作者(推定)</t>
         </is>
       </c>
       <c r="I402" t="inlineStr"/>
-      <c r="J402" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J402" t="inlineStr"/>
       <c r="K402" t="inlineStr"/>
       <c r="L402" t="inlineStr">
         <is>
-          <t>Faculty of Medicine and Institute of Clinical Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
+          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41364874</t>
         </is>
       </c>
       <c r="B403" t="n">
         <v>2026</v>
       </c>
       <c r="C403" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Chun-Ying Wu</t>
+          <t>Cho-Hao Lee</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>0000-0001-5053-1801</t>
+          <t>0000-0002-6061-5168</t>
         </is>
       </c>
       <c r="F403" t="inlineStr"/>
@@ -26655,88 +26559,76 @@
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>OpenAlex</t>
+          <t>末位作者(推定)</t>
         </is>
       </c>
       <c r="I403" t="inlineStr"/>
-      <c r="J403" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J403" t="inlineStr"/>
       <c r="K403" t="inlineStr"/>
       <c r="L403" t="inlineStr">
         <is>
-          <t>Institute of Biomedical Informatics, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
+          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41252340</t>
         </is>
       </c>
       <c r="B404" t="n">
         <v>2026</v>
       </c>
       <c r="C404" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>Chun-Ying Wu</t>
-        </is>
-      </c>
-      <c r="E404" t="inlineStr">
-        <is>
-          <t>0000-0001-5053-1801</t>
-        </is>
-      </c>
-      <c r="F404" t="inlineStr"/>
-      <c r="G404" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H404" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+          <t>Tai-Yung Yi</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr"/>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr"/>
+      <c r="H404" t="inlineStr"/>
       <c r="I404" t="inlineStr"/>
-      <c r="J404" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K404" t="inlineStr"/>
+      <c r="J404" t="inlineStr"/>
+      <c r="K404" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>Division of Translational Research, Taipei Veterans General Hospital, Taipei, Taiwan.</t>
+          <t>Department of Pharmacy, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>41105233</t>
+          <t>41252340</t>
         </is>
       </c>
       <c r="B405" t="n">
         <v>2026</v>
       </c>
       <c r="C405" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Chun-Ying Wu</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>0000-0001-5053-1801</t>
+          <t>0000-0002-9458-5665</t>
         </is>
       </c>
       <c r="F405" t="inlineStr"/>
@@ -26747,114 +26639,110 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>OpenAlex</t>
+          <t>PubMed e-mail</t>
         </is>
       </c>
       <c r="I405" t="inlineStr"/>
-      <c r="J405" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K405" t="inlineStr"/>
+      <c r="J405" t="inlineStr"/>
+      <c r="K405" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>College of Public Health, China Medical University, Taichung, Taiwan.</t>
+          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan, reillyjj@qut.edu.au.</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>41014190</t>
+          <t>41252340</t>
         </is>
       </c>
       <c r="B406" t="n">
         <v>2026</v>
       </c>
       <c r="C406" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Meing-Chung Chang</t>
-        </is>
-      </c>
-      <c r="E406" t="inlineStr"/>
-      <c r="F406" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G406" t="inlineStr"/>
-      <c r="H406" t="inlineStr"/>
+          <t>Joshua Wang</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>0000-0002-9458-5665</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr"/>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>PubMed e-mail</t>
+        </is>
+      </c>
       <c r="I406" t="inlineStr"/>
       <c r="J406" t="inlineStr"/>
-      <c r="K406" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K406" t="inlineStr"/>
       <c r="L406" t="inlineStr">
         <is>
-          <t>Department of Plastic Surgery, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City 231, Taiwan.</t>
+          <t>School of Biomedical Sciences, Queensland University of Technology, Brisbane, Queensland, Australia, reillyjj@qut.edu.au.</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>41014190</t>
+          <t>41242897</t>
         </is>
       </c>
       <c r="B407" t="n">
         <v>2026</v>
       </c>
       <c r="C407" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Hung-Da Chen</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
-        </is>
-      </c>
-      <c r="F407" t="inlineStr"/>
-      <c r="G407" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H407" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+          <t>0009-0000-0327-8663</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr"/>
+      <c r="H407" t="inlineStr"/>
       <c r="I407" t="inlineStr"/>
-      <c r="J407" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J407" t="inlineStr"/>
       <c r="K407" s="14" t="inlineStr">
         <is>
-          <t>台北慈濟醫院</t>
+          <t>台北慈濟醫院; 慈濟大學</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City 231, Taiwan.</t>
+          <t>Division of Gastroenterology, Department of Internal Medicine, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan; College of Medicine, Tzu Chi University, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>41014190</t>
+          <t>41242897</t>
         </is>
       </c>
       <c r="B408" t="n">
@@ -26890,17 +26778,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K408" t="inlineStr"/>
+      <c r="K408" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t>School of Biomedical Sciences, Queensland University of Technology, Brisbane 4000, Australia.</t>
+          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan; School of Biomedical Sciences, Queensland University of Technology, Brisbane, Australia. Electronic address: reillyjj@qut.edu.au.</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41167602</t>
         </is>
       </c>
       <c r="B409" t="n">
@@ -26911,12 +26803,12 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Tai-Li Chen</t>
+          <t>Chee-Seng Lee</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>0000-0002-5761-8114</t>
+          <t>0000-0002-3681-7288</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
@@ -26924,33 +26816,25 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G409" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H409" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+      <c r="G409" t="inlineStr"/>
+      <c r="H409" t="inlineStr"/>
       <c r="I409" t="inlineStr"/>
-      <c r="J409" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K409" t="inlineStr"/>
+      <c r="J409" t="inlineStr"/>
+      <c r="K409" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>Department of Dermatology, Taipei Veterans General Hospital, Taipei, Taiwan.</t>
+          <t>Department of Pediatrics, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41167602</t>
         </is>
       </c>
       <c r="B410" t="n">
@@ -26961,12 +26845,12 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>Tai-Li Chen</t>
+          <t>Chee-Seng Lee</t>
         </is>
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>0000-0002-5761-8114</t>
+          <t>0000-0002-3681-7288</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
@@ -26974,33 +26858,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G410" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H410" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+      <c r="G410" t="inlineStr"/>
+      <c r="H410" t="inlineStr"/>
       <c r="I410" t="inlineStr"/>
-      <c r="J410" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J410" t="inlineStr"/>
       <c r="K410" t="inlineStr"/>
       <c r="L410" t="inlineStr">
         <is>
-          <t>Faculty of Medicine, School of Medicine, National Yang Ming Chao Tung University, Taipei, Taiwan.</t>
+          <t>Department of Pediatrics, National Taiwan University Children's Hospital, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41167602</t>
         </is>
       </c>
       <c r="B411" t="n">
@@ -27011,10 +26883,14 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>Hou-Ren Tsai</t>
-        </is>
-      </c>
-      <c r="E411" t="inlineStr"/>
+          <t>Joshua Wang</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>0000-0002-9458-5665</t>
+        </is>
+      </c>
       <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr">
         <is>
@@ -27023,30 +26899,26 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>OpenAlex</t>
+          <t>末位作者(推定)</t>
         </is>
       </c>
       <c r="I411" t="inlineStr"/>
-      <c r="J411" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K411" s="18" t="inlineStr">
-        <is>
-          <t>花蓮慈濟醫院</t>
+      <c r="J411" t="inlineStr"/>
+      <c r="K411" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>Department of Ophthalmology, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
+          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41167602</t>
         </is>
       </c>
       <c r="B412" t="n">
@@ -27057,10 +26929,14 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Hou-Ren Tsai</t>
-        </is>
-      </c>
-      <c r="E412" t="inlineStr"/>
+          <t>Joshua Wang</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>0000-0002-9458-5665</t>
+        </is>
+      </c>
       <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
@@ -27069,120 +26945,116 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>OpenAlex</t>
+          <t>末位作者(推定)</t>
         </is>
       </c>
       <c r="I412" t="inlineStr"/>
-      <c r="J412" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K412" s="17" t="inlineStr">
-        <is>
-          <t>慈濟大學</t>
-        </is>
-      </c>
+      <c r="J412" t="inlineStr"/>
+      <c r="K412" t="inlineStr"/>
       <c r="L412" t="inlineStr">
         <is>
-          <t>School of Medicine, Tzu Chi University, Hualien, Taiwan.</t>
+          <t>School of Biomedical Sciences, Queensland University of Technology, Brisbane, Australia.</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B413" t="n">
         <v>2026</v>
       </c>
       <c r="C413" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Wei-Chuan Chang</t>
+          <t>Teng-Li Lin</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>0009-0009-8781-9708</t>
-        </is>
-      </c>
-      <c r="F413" t="inlineStr"/>
+          <t>0000-0002-0639-3533</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G413" t="inlineStr"/>
       <c r="H413" t="inlineStr"/>
       <c r="I413" t="inlineStr"/>
       <c r="J413" t="inlineStr"/>
-      <c r="K413" s="18" t="inlineStr">
-        <is>
-          <t>花蓮慈濟醫院</t>
+      <c r="K413" s="19" t="inlineStr">
+        <is>
+          <t>大林慈濟醫院</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t>Epidemiology and Biostatistics Center, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
+          <t>Department of Dermatology, Dalin Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Chiayi, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B414" t="n">
         <v>2026</v>
       </c>
       <c r="C414" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Jing-Wun Lu</t>
-        </is>
-      </c>
-      <c r="E414" t="inlineStr"/>
-      <c r="F414" t="inlineStr"/>
+          <t>Teng-Li Lin</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>0000-0002-0639-3533</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G414" t="inlineStr"/>
       <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr"/>
       <c r="J414" t="inlineStr"/>
-      <c r="K414" s="18" t="inlineStr">
-        <is>
-          <t>花蓮慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K414" t="inlineStr"/>
       <c r="L414" t="inlineStr">
         <is>
-          <t>Department of Physical Medicine and Rehabilitation, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
+          <t>Ph.D. Program of Interdisciplinary Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B415" t="n">
         <v>2026</v>
       </c>
       <c r="C415" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Yi-Ju Chen</t>
-        </is>
-      </c>
-      <c r="E415" t="inlineStr">
-        <is>
-          <t>0000-0001-5057-8060</t>
-        </is>
-      </c>
+          <t>Yi-Hsuan Fan</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr"/>
       <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr"/>
       <c r="H415" t="inlineStr"/>
@@ -27191,68 +27063,64 @@
       <c r="K415" t="inlineStr"/>
       <c r="L415" t="inlineStr">
         <is>
-          <t>Department of Dermatology, Taichung Veterans General Hospital, Taichung, Taiwan.</t>
+          <t>Department of Pediatrics, Chung Shan Medical University Hospital, Taichung, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B416" t="n">
         <v>2026</v>
       </c>
       <c r="C416" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Yuan-Chieh Lee</t>
-        </is>
-      </c>
-      <c r="E416" t="inlineStr">
-        <is>
-          <t>0000-0002-8486-8549</t>
-        </is>
-      </c>
+          <t>Kuo-Sheng Fan</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr"/>
       <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr"/>
       <c r="H416" t="inlineStr"/>
       <c r="I416" t="inlineStr"/>
       <c r="J416" t="inlineStr"/>
-      <c r="K416" s="18" t="inlineStr">
-        <is>
-          <t>花蓮慈濟醫院</t>
+      <c r="K416" s="19" t="inlineStr">
+        <is>
+          <t>大林慈濟醫院</t>
         </is>
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t>Department of Ophthalmology, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
+          <t>Division of Chest Medicine, Department of Internal Medicine, Dalin Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Chiayi, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B417" t="n">
         <v>2026</v>
       </c>
       <c r="C417" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Yuan-Chieh Lee</t>
+          <t>Chao-Kuei Juan</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>0000-0002-8486-8549</t>
+          <t>0000-0002-8846-0831</t>
         </is>
       </c>
       <c r="F417" t="inlineStr"/>
@@ -27260,529 +27128,669 @@
       <c r="H417" t="inlineStr"/>
       <c r="I417" t="inlineStr"/>
       <c r="J417" t="inlineStr"/>
-      <c r="K417" s="17" t="inlineStr">
-        <is>
-          <t>慈濟大學</t>
-        </is>
-      </c>
+      <c r="K417" t="inlineStr"/>
       <c r="L417" t="inlineStr">
         <is>
-          <t>Department of Ophthalmology and Visual Science, Tzu Chi University, Hualien, Taiwan.</t>
+          <t>Department of Dermatology, Taichung Veterans General Hospital, Taichung, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B418" t="n">
         <v>2026</v>
       </c>
       <c r="C418" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Chen-Yi Wu</t>
-        </is>
-      </c>
-      <c r="E418" t="inlineStr">
-        <is>
-          <t>0000-0002-8393-3900</t>
-        </is>
-      </c>
+          <t>Yi-Ju Chen</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr"/>
       <c r="F418" t="inlineStr"/>
-      <c r="G418" t="inlineStr"/>
-      <c r="H418" t="inlineStr"/>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I418" t="inlineStr"/>
-      <c r="J418" t="inlineStr"/>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K418" t="inlineStr"/>
       <c r="L418" t="inlineStr">
         <is>
-          <t>Department of Dermatology, Taipei Veterans General Hospital, Taipei, Taiwan.</t>
+          <t>Department of Dermatology, Taichung Veterans General Hospital, Taichung, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B419" t="n">
         <v>2026</v>
       </c>
       <c r="C419" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Chen-Yi Wu</t>
-        </is>
-      </c>
-      <c r="E419" t="inlineStr">
-        <is>
-          <t>0000-0002-8393-3900</t>
-        </is>
-      </c>
+          <t>Yi-Ju Chen</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr"/>
-      <c r="G419" t="inlineStr"/>
-      <c r="H419" t="inlineStr"/>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I419" t="inlineStr"/>
-      <c r="J419" t="inlineStr"/>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K419" t="inlineStr"/>
       <c r="L419" t="inlineStr">
         <is>
-          <t>Faculty of Medicine, School of Medicine, National Yang Ming Chao Tung University, Taipei, Taiwan.</t>
+          <t>Department of Post-Baccalaureate Medicine, National Chung-Hsing University, Taichung, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B420" t="n">
         <v>2026</v>
       </c>
       <c r="C420" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Chen-Yi Wu</t>
-        </is>
-      </c>
-      <c r="E420" t="inlineStr">
-        <is>
-          <t>0000-0002-8393-3900</t>
-        </is>
-      </c>
+          <t>Yi-Ju Chen</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr"/>
       <c r="F420" t="inlineStr"/>
-      <c r="G420" t="inlineStr"/>
-      <c r="H420" t="inlineStr"/>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I420" t="inlineStr"/>
-      <c r="J420" t="inlineStr"/>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K420" t="inlineStr"/>
       <c r="L420" t="inlineStr">
         <is>
-          <t>Faculty of Medicine and Institute of Clinical Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan; and.</t>
+          <t>Faculty of Medicine and Institute of Clinical Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>40729752</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B421" t="n">
         <v>2026</v>
       </c>
       <c r="C421" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Chen-Yi Wu</t>
+          <t>Chun-Ying Wu</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>0000-0002-8393-3900</t>
+          <t>0000-0001-5053-1801</t>
         </is>
       </c>
       <c r="F421" t="inlineStr"/>
-      <c r="G421" t="inlineStr"/>
-      <c r="H421" t="inlineStr"/>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I421" t="inlineStr"/>
-      <c r="J421" t="inlineStr"/>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K421" t="inlineStr"/>
       <c r="L421" t="inlineStr">
         <is>
-          <t>Department of Public Health, Institute of Public Health, National Yang Ming Chao Tung University, Taipei, Taiwan.</t>
+          <t>Faculty of Medicine and Institute of Clinical Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B422" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C422" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Min-Tser Liao</t>
+          <t>Chun-Ying Wu</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>0000-0002-7698-5331</t>
-        </is>
-      </c>
-      <c r="F422" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G422" t="inlineStr"/>
-      <c r="H422" t="inlineStr"/>
+          <t>0000-0001-5053-1801</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr"/>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I422" t="inlineStr"/>
-      <c r="J422" t="inlineStr"/>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K422" t="inlineStr"/>
       <c r="L422" t="inlineStr">
         <is>
-          <t>Department of Pediatrics, Taoyuan Armed Forces General Hospital, Taoyuan, Taiwan.</t>
+          <t>Institute of Biomedical Informatics, National Yang Ming Chiao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B423" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C423" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Min-Tser Liao</t>
+          <t>Chun-Ying Wu</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>0000-0002-7698-5331</t>
-        </is>
-      </c>
-      <c r="F423" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G423" t="inlineStr"/>
-      <c r="H423" t="inlineStr"/>
+          <t>0000-0001-5053-1801</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr"/>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I423" t="inlineStr"/>
-      <c r="J423" t="inlineStr"/>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K423" t="inlineStr"/>
       <c r="L423" t="inlineStr">
         <is>
-          <t>Department of Pediatrics, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Division of Translational Research, Taipei Veterans General Hospital, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>41105233</t>
         </is>
       </c>
       <c r="B424" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C424" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Chien-Lin Lu</t>
+          <t>Chun-Ying Wu</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>0000-0002-9452-5179</t>
+          <t>0000-0001-5053-1801</t>
         </is>
       </c>
       <c r="F424" t="inlineStr"/>
-      <c r="G424" t="inlineStr"/>
-      <c r="H424" t="inlineStr"/>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I424" t="inlineStr"/>
-      <c r="J424" t="inlineStr"/>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K424" t="inlineStr"/>
       <c r="L424" t="inlineStr">
         <is>
-          <t>School of Medicine, College of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
+          <t>College of Public Health, China Medical University, Taichung, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>41014190</t>
         </is>
       </c>
       <c r="B425" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C425" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Chien-Lin Lu</t>
-        </is>
-      </c>
-      <c r="E425" t="inlineStr">
-        <is>
-          <t>0000-0002-9452-5179</t>
-        </is>
-      </c>
-      <c r="F425" t="inlineStr"/>
+          <t>Meing-Chung Chang</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr"/>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G425" t="inlineStr"/>
       <c r="H425" t="inlineStr"/>
       <c r="I425" t="inlineStr"/>
       <c r="J425" t="inlineStr"/>
-      <c r="K425" t="inlineStr"/>
+      <c r="K425" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Medicine, Fu Jen Catholic University Hospital, New Taipei City, Taiwan.</t>
+          <t>Department of Plastic Surgery, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City 231, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>41014190</t>
         </is>
       </c>
       <c r="B426" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C426" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Yi-Chou Hou</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>0000-0001-7662-9890</t>
+          <t>0000-0002-9458-5665</t>
         </is>
       </c>
       <c r="F426" t="inlineStr"/>
-      <c r="G426" t="inlineStr"/>
-      <c r="H426" t="inlineStr"/>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I426" t="inlineStr"/>
-      <c r="J426" t="inlineStr"/>
-      <c r="K426" t="inlineStr"/>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K426" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L426" t="inlineStr">
         <is>
-          <t>School of Medicine, College of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
+          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City 231, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>41014190</t>
         </is>
       </c>
       <c r="B427" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C427" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Yi-Chou Hou</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>0000-0001-7662-9890</t>
+          <t>0000-0002-9458-5665</t>
         </is>
       </c>
       <c r="F427" t="inlineStr"/>
-      <c r="G427" t="inlineStr"/>
-      <c r="H427" t="inlineStr"/>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I427" t="inlineStr"/>
-      <c r="J427" t="inlineStr"/>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K427" t="inlineStr"/>
       <c r="L427" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Internal Medicine, Cardinal-Tien Hospital, School of Medicine, College of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
+          <t>School of Biomedical Sciences, Queensland University of Technology, Brisbane 4000, Australia.</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B428" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C428" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Tai-Li Chen</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>0009-0003-4519-2958</t>
-        </is>
-      </c>
-      <c r="F428" t="inlineStr"/>
-      <c r="G428" t="inlineStr"/>
-      <c r="H428" t="inlineStr"/>
+          <t>0000-0002-5761-8114</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I428" t="inlineStr"/>
-      <c r="J428" t="inlineStr"/>
-      <c r="K428" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr"/>
       <c r="L428" t="inlineStr">
         <is>
-          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>Department of Dermatology, Taipei Veterans General Hospital, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B429" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C429" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Kuo-Wang Tsai</t>
+          <t>Tai-Li Chen</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>0000-0002-9028-9834</t>
-        </is>
-      </c>
-      <c r="F429" t="inlineStr"/>
-      <c r="G429" t="inlineStr"/>
-      <c r="H429" t="inlineStr"/>
+          <t>0000-0002-5761-8114</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I429" t="inlineStr"/>
-      <c r="J429" t="inlineStr"/>
-      <c r="K429" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr"/>
       <c r="L429" t="inlineStr">
         <is>
-          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>Faculty of Medicine, School of Medicine, National Yang Ming Chao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B430" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C430" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Li-Jane Shih</t>
-        </is>
-      </c>
-      <c r="E430" t="inlineStr">
-        <is>
-          <t>0000-0001-7195-7676</t>
-        </is>
-      </c>
+          <t>Hou-Ren Tsai</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr"/>
-      <c r="G430" t="inlineStr"/>
-      <c r="H430" t="inlineStr"/>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I430" t="inlineStr"/>
-      <c r="J430" t="inlineStr"/>
-      <c r="K430" t="inlineStr"/>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K430" s="18" t="inlineStr">
+        <is>
+          <t>花蓮慈濟醫院</t>
+        </is>
+      </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t>Department of Medical Laboratory, Taoyuan Armed Forces General Hospital, Longtan, Taoyuan, Taiwan.</t>
+          <t>Department of Ophthalmology, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B431" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C431" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Li-Jane Shih</t>
-        </is>
-      </c>
-      <c r="E431" t="inlineStr">
-        <is>
-          <t>0000-0001-7195-7676</t>
-        </is>
-      </c>
+          <t>Hou-Ren Tsai</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr"/>
       <c r="F431" t="inlineStr"/>
-      <c r="G431" t="inlineStr"/>
-      <c r="H431" t="inlineStr"/>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I431" t="inlineStr"/>
-      <c r="J431" t="inlineStr"/>
-      <c r="K431" t="inlineStr"/>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K431" s="17" t="inlineStr">
+        <is>
+          <t>慈濟大學</t>
+        </is>
+      </c>
       <c r="L431" t="inlineStr">
         <is>
-          <t>Graduate Institute of Medical Science, National Defense Medical Center, Taipei, Taiwan.</t>
+          <t>School of Medicine, Tzu Chi University, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B432" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C432" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Chia-Chao Wu</t>
+          <t>Wei-Chuan Chang</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>0000-0002-8772-011X</t>
+          <t>0009-0009-8781-9708</t>
         </is>
       </c>
       <c r="F432" t="inlineStr"/>
@@ -27790,71 +27798,71 @@
       <c r="H432" t="inlineStr"/>
       <c r="I432" t="inlineStr"/>
       <c r="J432" t="inlineStr"/>
-      <c r="K432" t="inlineStr"/>
+      <c r="K432" s="18" t="inlineStr">
+        <is>
+          <t>花蓮慈濟醫院</t>
+        </is>
+      </c>
       <c r="L432" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical Center, Taipei, Taiwan.</t>
+          <t>Epidemiology and Biostatistics Center, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B433" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C433" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Yi-Chun Wang</t>
-        </is>
-      </c>
-      <c r="E433" t="inlineStr">
-        <is>
-          <t>0000-0002-5624-5571</t>
-        </is>
-      </c>
+          <t>Jing-Wun Lu</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr"/>
       <c r="H433" t="inlineStr"/>
       <c r="I433" t="inlineStr"/>
       <c r="J433" t="inlineStr"/>
-      <c r="K433" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
+      <c r="K433" s="18" t="inlineStr">
+        <is>
+          <t>花蓮慈濟醫院</t>
         </is>
       </c>
       <c r="L433" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Medicine, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>Department of Physical Medicine and Rehabilitation, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B434" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C434" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Yi-Chun Wang</t>
+          <t>Yi-Ju Chen</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>0000-0002-5624-5571</t>
+          <t>0000-0001-5057-8060</t>
         </is>
       </c>
       <c r="F434" t="inlineStr"/>
@@ -27862,187 +27870,143 @@
       <c r="H434" t="inlineStr"/>
       <c r="I434" t="inlineStr"/>
       <c r="J434" t="inlineStr"/>
-      <c r="K434" s="18" t="inlineStr">
-        <is>
-          <t>花蓮慈濟醫院; 慈濟大學</t>
-        </is>
-      </c>
+      <c r="K434" t="inlineStr"/>
       <c r="L434" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Medicine, Buddhist Tzu Chi University, Hualien, Taiwan.</t>
+          <t>Department of Dermatology, Taichung Veterans General Hospital, Taichung, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B435" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C435" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Kuo-Cheng Lu</t>
+          <t>Yuan-Chieh Lee</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>0000-0002-7062-8560</t>
+          <t>0000-0002-8486-8549</t>
         </is>
       </c>
       <c r="F435" t="inlineStr"/>
-      <c r="G435" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H435" t="inlineStr">
-        <is>
-          <t>PMC全文</t>
-        </is>
-      </c>
-      <c r="I435" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J435" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K435" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
+      <c r="G435" t="inlineStr"/>
+      <c r="H435" t="inlineStr"/>
+      <c r="I435" t="inlineStr"/>
+      <c r="J435" t="inlineStr"/>
+      <c r="K435" s="18" t="inlineStr">
+        <is>
+          <t>花蓮慈濟醫院</t>
         </is>
       </c>
       <c r="L435" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Medicine, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
+          <t>Department of Ophthalmology, Hualien Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>41445831</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B436" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C436" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Kuo-Cheng Lu</t>
+          <t>Yuan-Chieh Lee</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>0000-0002-7062-8560</t>
+          <t>0000-0002-8486-8549</t>
         </is>
       </c>
       <c r="F436" t="inlineStr"/>
-      <c r="G436" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H436" t="inlineStr">
-        <is>
-          <t>PMC全文</t>
-        </is>
-      </c>
-      <c r="I436" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J436" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K436" t="inlineStr"/>
+      <c r="G436" t="inlineStr"/>
+      <c r="H436" t="inlineStr"/>
+      <c r="I436" t="inlineStr"/>
+      <c r="J436" t="inlineStr"/>
+      <c r="K436" s="17" t="inlineStr">
+        <is>
+          <t>慈濟大學</t>
+        </is>
+      </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t>Division of Nephrology, Department of Medicine, Fu Jen Catholic University Hospital, School of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
+          <t>Department of Ophthalmology and Visual Science, Tzu Chi University, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>41427560</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B437" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C437" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Kuen-Huei Lin</t>
-        </is>
-      </c>
-      <c r="E437" t="inlineStr"/>
-      <c r="F437" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G437" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H437" t="inlineStr">
-        <is>
-          <t>OpenAlex</t>
-        </is>
-      </c>
+          <t>Chen-Yi Wu</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>0000-0002-8393-3900</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr"/>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr"/>
       <c r="I437" t="inlineStr"/>
-      <c r="J437" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J437" t="inlineStr"/>
       <c r="K437" t="inlineStr"/>
       <c r="L437" t="inlineStr">
         <is>
-          <t>Departments of Orthopedics.</t>
+          <t>Department of Dermatology, Taipei Veterans General Hospital, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>41427560</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B438" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C438" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Chen-Yi Wu</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
+          <t>0000-0002-8393-3900</t>
         </is>
       </c>
       <c r="F438" t="inlineStr"/>
@@ -28050,37 +28014,33 @@
       <c r="H438" t="inlineStr"/>
       <c r="I438" t="inlineStr"/>
       <c r="J438" t="inlineStr"/>
-      <c r="K438" s="14" t="inlineStr">
-        <is>
-          <t>台北慈濟醫院</t>
-        </is>
-      </c>
+      <c r="K438" t="inlineStr"/>
       <c r="L438" t="inlineStr">
         <is>
-          <t>Research, Taipei Tzu Chi Hospital Buddhist Tzu Chi Medical Foundation New Taipei City, Taiwan.</t>
+          <t>Faculty of Medicine, School of Medicine, National Yang Ming Chao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>41427560</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B439" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C439" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Joshua Wang</t>
+          <t>Chen-Yi Wu</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>0000-0002-9458-5665</t>
+          <t>0000-0002-8393-3900</t>
         </is>
       </c>
       <c r="F439" t="inlineStr"/>
@@ -28091,37 +28051,33 @@
       <c r="K439" t="inlineStr"/>
       <c r="L439" t="inlineStr">
         <is>
-          <t>School of Biomedical Sciences Queensland University of Technology Brisbane, QLD Australia.</t>
+          <t>Faculty of Medicine and Institute of Clinical Medicine, National Yang Ming Chiao Tung University, Taipei, Taiwan; and.</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>40729752</t>
         </is>
       </c>
       <c r="B440" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C440" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Ren-Hua Ye</t>
+          <t>Chen-Yi Wu</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>0000-0003-2418-7829</t>
-        </is>
-      </c>
-      <c r="F440" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>0000-0002-8393-3900</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr"/>
       <c r="G440" t="inlineStr"/>
       <c r="H440" t="inlineStr"/>
       <c r="I440" t="inlineStr"/>
@@ -28129,14 +28085,14 @@
       <c r="K440" t="inlineStr"/>
       <c r="L440" t="inlineStr">
         <is>
-          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Department of Public Health, Institute of Public Health, National Yang Ming Chao Tung University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B441" t="n">
@@ -28147,12 +28103,12 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Ren-Hua Ye</t>
+          <t>Min-Tser Liao</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>0000-0003-2418-7829</t>
+          <t>0000-0002-7698-5331</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
@@ -28167,33 +28123,37 @@
       <c r="K441" t="inlineStr"/>
       <c r="L441" t="inlineStr">
         <is>
-          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Department of Pediatrics, Taoyuan Armed Forces General Hospital, Taoyuan, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B442" t="n">
         <v>2025</v>
       </c>
       <c r="C442" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Hong-Jie Jhou</t>
+          <t>Min-Tser Liao</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>0000-0003-3304-4643</t>
-        </is>
-      </c>
-      <c r="F442" t="inlineStr"/>
+          <t>0000-0002-7698-5331</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G442" t="inlineStr"/>
       <c r="H442" t="inlineStr"/>
       <c r="I442" t="inlineStr"/>
@@ -28201,30 +28161,30 @@
       <c r="K442" t="inlineStr"/>
       <c r="L442" t="inlineStr">
         <is>
-          <t>Neurological Institute, Changhua Christian Hospital, Changhua, Taiwan.</t>
+          <t>Department of Pediatrics, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B443" t="n">
         <v>2025</v>
       </c>
       <c r="C443" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Hsin-Yu Chen</t>
+          <t>Chien-Lin Lu</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>0000-0002-2765-1685</t>
+          <t>0000-0002-9452-5179</t>
         </is>
       </c>
       <c r="F443" t="inlineStr"/>
@@ -28235,30 +28195,30 @@
       <c r="K443" t="inlineStr"/>
       <c r="L443" t="inlineStr">
         <is>
-          <t>Department of Family Medicine, Chi Mei Medical Center, Tainan, Taiwan.</t>
+          <t>School of Medicine, College of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B444" t="n">
         <v>2025</v>
       </c>
       <c r="C444" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Li-Ting Kao</t>
+          <t>Chien-Lin Lu</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>0000-0003-0692-7408</t>
+          <t>0000-0002-9452-5179</t>
         </is>
       </c>
       <c r="F444" t="inlineStr"/>
@@ -28269,30 +28229,30 @@
       <c r="K444" t="inlineStr"/>
       <c r="L444" t="inlineStr">
         <is>
-          <t>Graduate Institute of Life Sciences, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Medicine, Fu Jen Catholic University Hospital, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B445" t="n">
         <v>2025</v>
       </c>
       <c r="C445" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Li-Ting Kao</t>
+          <t>Yi-Chou Hou</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>0000-0003-0692-7408</t>
+          <t>0000-0001-7662-9890</t>
         </is>
       </c>
       <c r="F445" t="inlineStr"/>
@@ -28303,30 +28263,30 @@
       <c r="K445" t="inlineStr"/>
       <c r="L445" t="inlineStr">
         <is>
-          <t>School of Pharmacy, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>School of Medicine, College of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B446" t="n">
         <v>2025</v>
       </c>
       <c r="C446" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Li-Ting Kao</t>
+          <t>Yi-Chou Hou</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>0000-0003-0692-7408</t>
+          <t>0000-0001-7662-9890</t>
         </is>
       </c>
       <c r="F446" t="inlineStr"/>
@@ -28337,30 +28297,30 @@
       <c r="K446" t="inlineStr"/>
       <c r="L446" t="inlineStr">
         <is>
-          <t>Department of Pharmacy Practice, Tri-Service General Hospital, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Internal Medicine, Cardinal-Tien Hospital, School of Medicine, College of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B447" t="n">
         <v>2025</v>
       </c>
       <c r="C447" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Tina Yi-Jin Hsieh</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>0000-0001-6296-0689</t>
+          <t>0009-0003-4519-2958</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -28368,33 +28328,37 @@
       <c r="H447" t="inlineStr"/>
       <c r="I447" t="inlineStr"/>
       <c r="J447" t="inlineStr"/>
-      <c r="K447" t="inlineStr"/>
+      <c r="K447" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L447" t="inlineStr">
         <is>
-          <t>Department of Obstetrics and Gynecology, Beth Israel Deaconess Medical Center, Boston, MA.</t>
+          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B448" t="n">
         <v>2025</v>
       </c>
       <c r="C448" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Yu-Han Chen</t>
+          <t>Kuo-Wang Tsai</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>0000-0001-9170-7439</t>
+          <t>0000-0002-9028-9834</t>
         </is>
       </c>
       <c r="F448" t="inlineStr"/>
@@ -28402,33 +28366,37 @@
       <c r="H448" t="inlineStr"/>
       <c r="I448" t="inlineStr"/>
       <c r="J448" t="inlineStr"/>
-      <c r="K448" t="inlineStr"/>
+      <c r="K448" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L448" t="inlineStr">
         <is>
-          <t>Department of Internal Medicine, Englewood Hospital and Medical Center, Englewood, NJ.</t>
+          <t>Department of Research, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B449" t="n">
         <v>2025</v>
       </c>
       <c r="C449" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Xiaoyi Zhang</t>
+          <t>Li-Jane Shih</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>0000-0001-5124-4919</t>
+          <t>0000-0001-7195-7676</t>
         </is>
       </c>
       <c r="F449" t="inlineStr"/>
@@ -28439,30 +28407,30 @@
       <c r="K449" t="inlineStr"/>
       <c r="L449" t="inlineStr">
         <is>
-          <t>Department of Internal Medicine, NYC Health + Hospitals/Jacobi, Albert Einstein College of Medicine, Bronx, NY.</t>
+          <t>Department of Medical Laboratory, Taoyuan Armed Forces General Hospital, Longtan, Taoyuan, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B450" t="n">
         <v>2025</v>
       </c>
       <c r="C450" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Ming-Shen Dai</t>
+          <t>Li-Jane Shih</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>0000-0002-3953-5243</t>
+          <t>0000-0001-7195-7676</t>
         </is>
       </c>
       <c r="F450" t="inlineStr"/>
@@ -28473,30 +28441,30 @@
       <c r="K450" t="inlineStr"/>
       <c r="L450" t="inlineStr">
         <is>
-          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Graduate Institute of Medical Science, National Defense Medical Center, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B451" t="n">
         <v>2025</v>
       </c>
       <c r="C451" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Ming-Shen Dai</t>
+          <t>Chia-Chao Wu</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>0000-0002-3953-5243</t>
+          <t>0000-0002-8772-011X</t>
         </is>
       </c>
       <c r="F451" t="inlineStr"/>
@@ -28507,30 +28475,30 @@
       <c r="K451" t="inlineStr"/>
       <c r="L451" t="inlineStr">
         <is>
-          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical Center, Taipei, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B452" t="n">
         <v>2025</v>
       </c>
       <c r="C452" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Ching-Liang Ho</t>
+          <t>Yi-Chun Wang</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>0000-0002-8378-1687</t>
+          <t>0000-0002-5624-5571</t>
         </is>
       </c>
       <c r="F452" t="inlineStr"/>
@@ -28538,33 +28506,37 @@
       <c r="H452" t="inlineStr"/>
       <c r="I452" t="inlineStr"/>
       <c r="J452" t="inlineStr"/>
-      <c r="K452" t="inlineStr"/>
+      <c r="K452" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L452" t="inlineStr">
         <is>
-          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Medicine, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B453" t="n">
         <v>2025</v>
       </c>
       <c r="C453" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Ching-Liang Ho</t>
+          <t>Yi-Chun Wang</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>0000-0002-8378-1687</t>
+          <t>0000-0002-5624-5571</t>
         </is>
       </c>
       <c r="F453" t="inlineStr"/>
@@ -28572,17 +28544,21 @@
       <c r="H453" t="inlineStr"/>
       <c r="I453" t="inlineStr"/>
       <c r="J453" t="inlineStr"/>
-      <c r="K453" t="inlineStr"/>
+      <c r="K453" s="18" t="inlineStr">
+        <is>
+          <t>花蓮慈濟醫院; 慈濟大學</t>
+        </is>
+      </c>
       <c r="L453" t="inlineStr">
         <is>
-          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Medicine, Buddhist Tzu Chi University, Hualien, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B454" t="n">
@@ -28593,19 +28569,35 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Ching-Liang Ho</t>
+          <t>Kuo-Cheng Lu</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>0000-0002-8378-1687</t>
+          <t>0000-0002-7062-8560</t>
         </is>
       </c>
       <c r="F454" t="inlineStr"/>
-      <c r="G454" t="inlineStr"/>
-      <c r="H454" t="inlineStr"/>
-      <c r="I454" t="inlineStr"/>
-      <c r="J454" t="inlineStr"/>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>PMC全文</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K454" s="14" t="inlineStr">
         <is>
           <t>台北慈濟醫院</t>
@@ -28613,159 +28605,175 @@
       </c>
       <c r="L454" t="inlineStr">
         <is>
-          <t>Division of Hematology and Oncology, Medical Department, Taipei Tzu Chi Hospital, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Medicine, Taipei Tzu Chi Hospital, Buddhist Tzu Chi Medical Foundation, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41445831</t>
         </is>
       </c>
       <c r="B455" t="n">
         <v>2025</v>
       </c>
       <c r="C455" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Po-Huang Chen</t>
+          <t>Kuo-Cheng Lu</t>
         </is>
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>0000-0002-0280-6417</t>
+          <t>0000-0002-7062-8560</t>
         </is>
       </c>
       <c r="F455" t="inlineStr"/>
-      <c r="G455" t="inlineStr"/>
-      <c r="H455" t="inlineStr"/>
-      <c r="I455" t="inlineStr"/>
-      <c r="J455" t="inlineStr"/>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>PMC全文</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K455" t="inlineStr"/>
       <c r="L455" t="inlineStr">
         <is>
-          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Division of Nephrology, Department of Medicine, Fu Jen Catholic University Hospital, School of Medicine, Fu Jen Catholic University, New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41427560</t>
         </is>
       </c>
       <c r="B456" t="n">
         <v>2025</v>
       </c>
       <c r="C456" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>Po-Huang Chen</t>
-        </is>
-      </c>
-      <c r="E456" t="inlineStr">
-        <is>
-          <t>0000-0002-0280-6417</t>
-        </is>
-      </c>
-      <c r="F456" t="inlineStr"/>
-      <c r="G456" t="inlineStr"/>
-      <c r="H456" t="inlineStr"/>
+          <t>Kuen-Huei Lin</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr"/>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>OpenAlex</t>
+        </is>
+      </c>
       <c r="I456" t="inlineStr"/>
-      <c r="J456" t="inlineStr"/>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K456" t="inlineStr"/>
       <c r="L456" t="inlineStr">
         <is>
-          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Departments of Orthopedics.</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41427560</t>
         </is>
       </c>
       <c r="B457" t="n">
         <v>2025</v>
       </c>
       <c r="C457" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>Cho-Hao Lee</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>0000-0002-6061-5168</t>
+          <t>0000-0002-9458-5665</t>
         </is>
       </c>
       <c r="F457" t="inlineStr"/>
-      <c r="G457" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H457" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
-        </is>
-      </c>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr"/>
       <c r="I457" t="inlineStr"/>
       <c r="J457" t="inlineStr"/>
-      <c r="K457" t="inlineStr"/>
+      <c r="K457" s="14" t="inlineStr">
+        <is>
+          <t>台北慈濟醫院</t>
+        </is>
+      </c>
       <c r="L457" t="inlineStr">
         <is>
-          <t>Division of Hematology and Oncology, Department of Internal Medicine, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>Research, Taipei Tzu Chi Hospital Buddhist Tzu Chi Medical Foundation New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>41364874</t>
+          <t>41427560</t>
         </is>
       </c>
       <c r="B458" t="n">
         <v>2025</v>
       </c>
       <c r="C458" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>Cho-Hao Lee</t>
+          <t>Joshua Wang</t>
         </is>
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>0000-0002-6061-5168</t>
+          <t>0000-0002-9458-5665</t>
         </is>
       </c>
       <c r="F458" t="inlineStr"/>
-      <c r="G458" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H458" t="inlineStr">
-        <is>
-          <t>末位作者(推定)</t>
-        </is>
-      </c>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr"/>
       <c r="I458" t="inlineStr"/>
       <c r="J458" t="inlineStr"/>
       <c r="K458" t="inlineStr"/>
       <c r="L458" t="inlineStr">
         <is>
-          <t>Department of Oncology, Tri-Service General Hospital, National Defense Medical University, Taipei, Taiwan.</t>
+          <t>School of Biomedical Sciences Queensland University of Technology Brisbane, QLD Australia.</t>
         </is>
       </c>
     </row>
@@ -41627,67 +41635,67 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E382" r:id="rId275"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E383" r:id="rId276"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E384" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E386" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E387" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E388" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E389" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E390" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E391" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E392" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E393" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E394" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E395" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E398" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E402" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E403" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E404" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E405" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E407" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E408" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E409" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E410" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E413" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E415" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E416" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E417" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E418" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E419" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E420" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E421" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E422" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E423" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E424" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E425" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E426" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E427" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E428" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E429" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E430" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E431" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E432" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E433" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E385" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E386" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E387" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E388" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E389" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E390" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E391" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E392" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E393" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E394" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E395" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E396" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E397" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E398" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E399" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E400" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E401" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E402" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E403" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E405" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E406" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E407" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E408" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E409" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E410" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E411" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E412" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E413" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E414" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E417" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E421" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E422" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E423" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E424" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E426" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E427" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E428" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E429" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E432" r:id="rId316"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E434" r:id="rId317"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E435" r:id="rId318"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E436" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E438" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E439" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E440" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E441" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E442" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E443" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E444" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E445" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E446" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E447" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E448" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E449" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E450" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E451" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E452" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E453" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E454" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E455" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E456" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E437" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E438" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E439" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E440" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E441" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E442" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E443" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E444" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E445" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E446" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E447" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E448" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E449" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E450" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E451" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E452" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E453" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E454" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E455" r:id="rId338"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E457" r:id="rId339"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E458" r:id="rId340"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E459" r:id="rId341"/>
@@ -42078,10 +42086,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F4" t="n">
         <v>68</v>

</xml_diff>